<commit_message>
feat(drive-sync): add Azerbaijani phonetic transliteration matcher and consolidate duplicate folders
</commit_message>
<xml_diff>
--- a/.agents/skills/academic-drive-project-organizer/references/MASTER_PROJECT_CATALOG.xlsx
+++ b/.agents/skills/academic-drive-project-organizer/references/MASTER_PROJECT_CATALOG.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,52 +417,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Duzen ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Project Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Client Name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Total Price (M Tomans)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Paid (Tomans)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Matched Drive Folder</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Linked to Drive</t>
         </is>
@@ -515,7 +503,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Model 3</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J2" t="b">
@@ -721,11 +709,11 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Not linked</t>
+          <t>[My Work] Fatemeh Solati</t>
         </is>
       </c>
       <c r="J7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -805,11 +793,11 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Not linked</t>
+          <t>[My Work] Nafiseh Rajabiyan</t>
         </is>
       </c>
       <c r="J9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -889,7 +877,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Model Data 12</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J11" t="b">
@@ -931,7 +919,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Model Data 11</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J12" t="b">
@@ -973,7 +961,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>[Finished Works] Fateme Niknam</t>
+          <t>[My Work] Fateme Niknam</t>
         </is>
       </c>
       <c r="J13" t="b">
@@ -1013,7 +1001,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Model Data 16</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J14" t="b">
@@ -1179,11 +1167,11 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Not linked</t>
+          <t>[My Work] Səmaneh Firuzi</t>
         </is>
       </c>
       <c r="J18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1219,7 +1207,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Amiri</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J19" t="b">
@@ -1261,7 +1249,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Amiri</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J20" t="b">
@@ -1387,7 +1375,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Model Data 2</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J23" t="b">
@@ -1427,7 +1415,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Amiri</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J24" t="b">
@@ -1511,7 +1499,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Amiri</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J26" t="b">
@@ -1553,7 +1541,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Model Data 18</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J27" t="b">
@@ -1595,7 +1583,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Amiri</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J28" t="b">
@@ -1637,7 +1625,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>[Finished Works] Varesi</t>
+          <t>[My Work] Varesi</t>
         </is>
       </c>
       <c r="J29" t="b">
@@ -1679,7 +1667,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Model Data 13</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J30" t="b">
@@ -1721,7 +1709,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Amiri</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J31" t="b">
@@ -1889,11 +1877,11 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Not linked</t>
+          <t>[My Work] Sajad</t>
         </is>
       </c>
       <c r="J35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -2139,7 +2127,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Manova Data 3</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J41" t="b">
@@ -2181,7 +2169,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>[Finished Works] Kashi</t>
+          <t>[My Work] Kaşı</t>
         </is>
       </c>
       <c r="J42" t="b">
@@ -2223,7 +2211,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>[Pending Works] Marziyeh Sinayi</t>
+          <t>[My Work] Marziyeh Sinayi</t>
         </is>
       </c>
       <c r="J43" t="b">
@@ -2431,7 +2419,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Amiri</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J48" t="b">
@@ -2513,7 +2501,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>[Pending Works] Shahram Amiri</t>
+          <t>[My Work] Shahram Amiri Soldiers Data</t>
         </is>
       </c>
       <c r="J50" t="b">
@@ -2595,11 +2583,11 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Not linked</t>
+          <t>[My Work] Əlireza Baneşı</t>
         </is>
       </c>
       <c r="J52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>